<commit_message>
chore: update test evidence and reports for ABDM functional testing M2
</commit_message>
<xml_diff>
--- a/abdm-ft/final/M2_BUILDING_HIP_TEST_CASES.xlsx
+++ b/abdm-ft/final/M2_BUILDING_HIP_TEST_CASES.xlsx
@@ -858,19 +858,19 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Test Executed by: Clinicx tester (Ocimum Dentistry front desk)</t>
+          <t>Test Executed by: Manikanta N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Application/ System Name: Clinicx HMIS (web)</t>
+          <t>Application/ System Name: ClinicX (Yira Health Tech) - HIP IN3610001937 Ocimum dentistry; backend 85ae1bd, frontend ab5a8a0</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Test Execution date: 2026-10-27</t>
+          <t>Test Execution date: 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       <c r="J10" s="14" t="n"/>
       <c r="K10" s="14" t="inlineStr">
         <is>
-          <t>Screen: ABDM Records lists care contexts holding all 8 HI types (OP consultation, Prescription, Diagnostic report, Discharge summary, Immunization record, Health document, Wellness record, Invoice); View shows the FHIR-built records</t>
+          <t>Screen: ABDM Records for the group 2 patient: '26 records:' '26 linked to abha', HI type tags for all 8 (OP consultation, Prescription, Invoice, Immunization record, Wellness record, Health document, Diagnostic report, Discharge summary); View on OP-342 shows what the PHR app receives</t>
         </is>
       </c>
       <c r="L10" s="14" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="N10" s="14" t="inlineStr">
         <is>
-          <t>Each HI type is an NRCES document bundle stored against a care context (OP-342, DR-1, WR-2, IM-1, IP-4). Clinical elements carry SNOMED CT and LOINC codes; a prescription saved in this run codes the medicine as SNOMED CT 323510009. Evidence 01-10.</t>
+          <t>Build 85ae1bd, Provider login. Each HI type is an NRCES document bundle (Bundle.type document, Composition first; profiles OPConsultRecord, PrescriptionRecord, InvoiceRecord, ImmunizationRecord, WellnessRecord, HealthDocumentRecord, DiagnosticReportRecord, DischargeSummaryRecord) stored against a care context. SNOMED CT / LOINC codings: OP-347 OPConsultation 24, Prescription 8, ImmunizationRecord 4; DR-1 DiagnosticReport 3 (LOINC); WR-4 WellnessRecord 6 (LOINC); IP-4 DischargeSummary 12; DOC-127 HealthDocumentRecord 3; Invoice 0 (billing codes, as the InvoiceRecord profile binds). Evidence 1-3.</t>
         </is>
       </c>
       <c r="O10" s="14" t="inlineStr">
@@ -1189,7 +1189,7 @@
       <c r="J13" s="15" t="n"/>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>generate-token 202 (2aa13a9d-a040-45e5-b288-842609b83db8); on-generate-token linkToken present, response.requestId matched, abhaAddress xxx0319@sbx; next link 7f5e46e6-94a9-4b51-80e9-cfaf1cf242bb used the stored token, no new generate-token</t>
+          <t>generate-token 202 (00c8e3d1-4aa8-4e21-937f-fe692f88708a); on-generate-token linkToken present, response.requestId matched, abhaAddress xxx0319@sbx; next link 47926fe3-8e13-4b75-ab53-b9b5baceed3a used the stored token, no new generate-token</t>
         </is>
       </c>
       <c r="L13" s="16" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="N13" s="16" t="inlineStr">
         <is>
-          <t>No valid token held (cleared before the run): a prescription save requested one, stored against the patient and address for six months (expires 2027-04-28). A wellness record saved next linked with no second token request. Screen: WR-3 Linked to ABHA. Steps: 1 PASS (token requested and received, requestId matched); 2 PASS (stored against patient and ABHA address, 6 months); 3 PASS (reused, no second generate-token)</t>
+          <t>No valid token held (cleared before the case at the tester's request): a prescription saved in the UI requested one, stored against the patient and address for six months (expires 2027-04-29). A wellness record saved next (WR-5) linked with no second token request: 0 generate-token after 00c8e3d1; one stored token. Screen: RX-D7CD5098 and WR-5 'Linked to ABHA'. Evidence 1-3. Steps: 1 PASS (token requested and received, requestId matched); 2 PASS (stored against patient and ABHA address, 6 months); 3 PASS (reused for WR-5, no second generate-token)</t>
         </is>
       </c>
       <c r="O13" s="54" t="inlineStr">
@@ -1269,16 +1269,20 @@
       <c r="J14" s="15" t="n"/>
       <c r="K14" s="15" t="inlineStr">
         <is>
-          <t>link/carecontext 202 (f3416e5d-1884-4879-8b84-944dd1a1c054), on_carecontext 'Successfully Linked care context'; link/context/notify 202 (98a9f16f-7236-4aa8-b874-391b38932a86), on-notify acknowledgement SUCCESS</t>
-        </is>
-      </c>
-      <c r="L14" s="14" t="inlineStr"/>
+          <t>link/carecontext 202 on save (eb698f25-663b-46ca-9e84-6ef145db724f, 47926fe3-8e13-4b75-ab53-b9b5baceed3a), on_carecontext 'Successfully Linked care context'; link/context/notify 202 (800ed08d-86d7-46b8-8fd5-aed664ab5b4c), on-notify acknowledgement.status SUCCESS; PHR app shows the linked records</t>
+        </is>
+      </c>
+      <c r="L14" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="M14" s="14" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="18" t="inlineStr">
         <is>
-          <t>Needs tester: Needs tester: PHR app pull and screenshot (sheet step 2), asked at readiness and at the case; the tester cannot pull records in the PHR app in this run. Linking ran automatically on save with no click. Steps: 1 PASS (link initiated with the token on save, Successfully Linked care context); 2 needs tester (PHR app pull (tester cannot in this run), context notify SUCCESS observed)</t>
+          <t>Linking ran automatically on save with no click (prescription RX-D7CD5098, wellness WR-5). A consultation record (Toothache, Pulpitis) added to the linked visit OP-344 sent the context notify on its own (OPConsultation added to Invoice). PHR app (tester's screenshots phr-1..4): Amoxicillin prescription, wellness record, OP-344 consultation report from Ocimum dentistry; transfers 51-53 DELIVERED. Extra check (count mismatch, ABDM-1037) not run: no screen sends it. Evidence 1-2, phr-1..4. Steps: 1 PASS (link initiated with the token on save, Successfully Linked care context); 2 PASS (records pulled and visible in the PHR app (tester screenshots), context notify SUCCESS)</t>
         </is>
       </c>
       <c r="O14" s="55" t="n"/>
@@ -1320,14 +1324,22 @@
         </is>
       </c>
       <c r="J15" s="15" t="n"/>
-      <c r="K15" s="15" t="inlineStr"/>
-      <c r="L15" s="14" t="inlineStr"/>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>PHR app (tester): Ocimum dentistry Health Record pages for the Prescription record (Amoxicillin 500 mg oral capsule, Dental caries, 28 Oct 2026 06:50 PM), the Wellness record (BP 122/78, heart rate 72, 36.8 C, height 172 cm, weight 68 kg, BMI 23) and the Clinical consultation report of 27 Oct (Toothache, Pulpitis)</t>
+        </is>
+      </c>
+      <c r="L15" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="M15" s="14" t="n">
         <v>1</v>
       </c>
       <c r="N15" s="14" t="inlineStr">
         <is>
-          <t>Needs tester: Needs tester: PHR app 'Pull Records' for Ocimum dentistry and a screenshot, asked at the case; the tester cannot pull records in the PHR app in this run.</t>
+          <t>The care contexts linked in HIP_INTI_LINK_504/505 were pulled into the PHR app: health-information requests 2dbace9a, 1534304c, a535f7b1 answered, transfers 51 (RX-D7CD5098), 52 (WR-5), 53 (OP-344) DELIVERED. Evidence phr-1..4.</t>
         </is>
       </c>
       <c r="O15" s="56" t="n"/>
@@ -1401,10 +1413,24 @@
 If the patient is already registered in the HMIS with valid ABHA details, the system should automatically link the generated health records to the patient's ABHA through the HIP-Initiated Linking workflow, eliminating the need for User-Initiated Linking.</t>
         </is>
       </c>
-      <c r="K17" s="24" t="n"/>
-      <c r="L17" s="14" t="n"/>
-      <c r="M17" s="14" t="n"/>
-      <c r="N17" s="14" t="n"/>
+      <c r="K17" s="24" t="inlineStr">
+        <is>
+          <t>Tester logged in to the ABDM sandbox PHR app with the second ABHA (mobile ending 5506); the PHR app then searched, discovered and linked (discover 17df06aa-b95d-4f33-b2d0-5ba9cbf0677b from that login)</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="14" t="inlineStr">
+        <is>
+          <t>Human step, confirmed by the tester; the discover that follows carries the logged-in ABHA's verified identifiers.</t>
+        </is>
+      </c>
       <c r="O17" s="57" t="inlineStr">
         <is>
           <r>
@@ -1466,10 +1492,24 @@
         </is>
       </c>
       <c r="J18" s="14" t="n"/>
-      <c r="K18" s="14" t="n"/>
-      <c r="L18" s="14" t="n"/>
-      <c r="M18" s="14" t="n"/>
-      <c r="N18" s="14" t="n"/>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>PHR app 'Link My Health Records': search 'ocimum' -&gt; 'Hospitals matching your search': 'Ocimum dentistry' (phr-1.png); selecting it sent the discover to IN3610001937</t>
+        </is>
+      </c>
+      <c r="L18" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="14" t="inlineStr">
+        <is>
+          <t>Facility found and selected under Link New facility. Evidence phr-1.png.</t>
+        </is>
+      </c>
       <c r="O18" s="55" t="n"/>
     </row>
     <row r="19" ht="125.4" customHeight="1">
@@ -1511,10 +1551,24 @@
         </is>
       </c>
       <c r="J19" s="14" t="n"/>
-      <c r="K19" s="14" t="n"/>
-      <c r="L19" s="14" t="n"/>
-      <c r="M19" s="14" t="n"/>
-      <c r="N19" s="14" t="n"/>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>Inbound POST /api/v3/hip/patient/care-context/discover REQUEST-ID 17df06aa-b95d-4f33-b2d0-5ba9cbf0677b at 23:24:10 IST: transactionId f3c99f71-3824-4f30-8a2b-afc473b1f443 present, patient.id present, patient.verifiedIdentifiers [MOBILE, ABHA_NUMBER, abhaAddress], gender F, yearOfBirth 2004</t>
+        </is>
+      </c>
+      <c r="L19" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M19" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="14" t="inlineStr">
+        <is>
+          <t>The profile reached the HIP through the bridge; the HIP searched on the verified mobile and narrowed by name, gender and year of birth. Earlier discovers 4901885a (19:17), 1b6398a2 (19:39) and 96b633bd (20:16) also arrived; 71823539 (21:06) got ABDM 'Runtime Error' on our reply.</t>
+        </is>
+      </c>
       <c r="O19" s="55" t="n"/>
     </row>
     <row r="20" ht="26" customHeight="1">
@@ -1554,10 +1608,24 @@
         </is>
       </c>
       <c r="J20" s="16" t="n"/>
-      <c r="K20" s="16" t="n"/>
-      <c r="L20" s="16" t="n"/>
-      <c r="M20" s="16" t="n"/>
-      <c r="N20" s="16" t="n"/>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>Matched by MOBILE to patient OCM123-2026-0013 (registered without ABHA; Female, born 2004, mobile ending 5506); on-discover sent with matchedBy [MOBILE] and patient[].careContexts [RX-67209C38-D094-4EB0-B928-A13D4529CF57], accepted by ABDM; the PHR app showed that record under our patient reference (USER_INIT_LINK_604/phr-1.png)</t>
+        </is>
+      </c>
+      <c r="L20" s="16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" s="16" t="inlineStr">
+        <is>
+          <t>Screen check: the matched patient's mobile, gender (F) and year of birth (2004) agree with the discover's. The build does not store outbound reply bodies: the on-discover content is shown by the PHR screen and by the init that selected from it.</t>
+        </is>
+      </c>
       <c r="O20" s="55" t="n"/>
     </row>
     <row r="21" ht="26" customHeight="1">
@@ -1597,10 +1665,24 @@
         </is>
       </c>
       <c r="J21" s="16" t="n"/>
-      <c r="K21" s="16" t="n"/>
-      <c r="L21" s="16" t="n"/>
-      <c r="M21" s="16" t="n"/>
-      <c r="N21" s="16" t="n"/>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>PHR app 'We found the following details': the patient, 'RX-67209C38-D094-4EB0-B928-A13D4529CF57', 'Prescription, 28 Oct 2026' (phr-1.png); the person selected it: inbound link init 764fd0a5-cd3f-4b0d-8e1c-038a56341033 with transactionId f3c99f71 (equal to the discover's) and careContexts [RX-67209C38]</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M21" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="16" t="inlineStr">
+        <is>
+          <t>Only unlinked care contexts were offered (RX-3FBA9ECC, linked earlier, was not). Evidence phr-1.png.</t>
+        </is>
+      </c>
       <c r="O21" s="55" t="n"/>
     </row>
     <row r="22" ht="59.4" customHeight="1">
@@ -1643,10 +1725,24 @@
         </is>
       </c>
       <c r="J22" s="16" t="n"/>
-      <c r="K22" s="16" t="n"/>
-      <c r="L22" s="16" t="n"/>
-      <c r="M22" s="16" t="n"/>
-      <c r="N22" s="16" t="n"/>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>init 764fd0a5-cd3f-4b0d-8e1c-038a56341033 (transactionId f3c99f71, selected RX-67209C38) -&gt; on-init with link.referenceNumber a402340b-c3d4-420f-88bb-26b0ca563e4d, authenticationType DIRECT, communicationMedium MOBILE, accepted; OTP sent by the HIP (ClinicX SMS) to the mobile ending 5506; confirm 44b6d7d6-9720-4573-b350-b65c8cf57e9d with confirmation.linkRefNumber a402340b and token present -&gt; OTP verified, on-confirm with RX-67209C38 only, accepted; care context linked via patient to xxx0606@sbx</t>
+        </is>
+      </c>
+      <c r="L22" s="16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M22" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>Link request 5 is created only after the OTP SMS is sent; it closed 'linked' at confirm (attempts 0). Screen check: the linked record shows under Ocimum dentistry in the PHR app (phr-3-linked-record.png: Prescription record, Acetaminophen 500 mg, Authored 28 Oct 2026 08:08 PM). Evidence phr-1 (records found), phr-3. Extra check (wrong OTP) not run. Steps: 1 PASS (init received, on-init DIRECT/MOBILE with link reference); 2 PASS (OTP sent by the HIP, confirm with matching linkRefNumber and token); 3 PASS (on-confirm with the selected care context only, record visible under the linked facility)</t>
+        </is>
+      </c>
       <c r="O22" s="55" t="n"/>
     </row>
     <row r="23" ht="26" customHeight="1">
@@ -1687,10 +1783,24 @@
         </is>
       </c>
       <c r="J23" s="16" t="n"/>
-      <c r="K23" s="16" t="n"/>
-      <c r="L23" s="16" t="n"/>
-      <c r="M23" s="16" t="n"/>
-      <c r="N23" s="16" t="n"/>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>Pull Records in the PHR app (mobile 5506): consent 28485736-f920-4444-b9a5-a2d7d5e24af2 for RX-67209C38 -&gt; HI request 20ae5b76-ded9-4738-8b0f-5a46676b28a5 -&gt; transfer 58 RX-67209C38 DELIVERED; PHR shows 'Prescription record' 'Acetaminophen 500 mg oral tablet' 'Gingivitis' 'Authored Date: 28 Oct 2026, 08:08 PM'</t>
+        </is>
+      </c>
+      <c r="L23" s="16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M23" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>Passes 1 (23:25) and 2 (23:33): the PHR app granted consents b0c64ca9 and 83f32143 for RX-67209C38 and the HIP acknowledged them, but ABDM sent no health-information request, so nothing could be pushed. Pass 3 (23:56, deferred to the end at the tester's request) delivered it. Evidence phr-1.png.</t>
+        </is>
+      </c>
       <c r="O23" s="56" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
@@ -1804,10 +1914,24 @@
         </is>
       </c>
       <c r="J25" s="14" t="n"/>
-      <c r="K25" s="14" t="n"/>
-      <c r="L25" s="14" t="n"/>
-      <c r="M25" s="14" t="n"/>
-      <c r="N25" s="14" t="n"/>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>sms/notify2 202 (ee33aa71-2e46-4704-8472-d823408f26bf), sent on save with no click; callback /api/v3/patients/sms/on-notify {"status":"ACKNOWLEDGED","error":null} with response.requestId matched; SMS from AD-NHASMS-S received on the mobile ending 5506: 'Your Ocimum dentistry reports are now ready ... https://phrsbx.abdm.gov.in/phr/v3/uhi?hipId=IN3610001937'</t>
+        </is>
+      </c>
+      <c r="L25" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M25" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="14" t="inlineStr">
+        <is>
+          <t>A prescription (Acetaminophen 500 mg oral tablet, Gingivitis) saved for patient OCM123-2026-0013, registered with a mobile and no ABHA address, sent the SMS notify on its own. The sandbox answers with status ACKNOWLEDGED and no error, which means the same as the acknowledgement.status SUCCESS the skill names. Tester's SMS screenshot kept with the earlier OTP messages blacked out (sms.png). Evidence 1, sms.png.</t>
+        </is>
+      </c>
       <c r="O25" s="23" t="inlineStr">
         <is>
           <t>https://dev.abdm.gov.in/api/hiecm/hip/v3/link/patient/links/sms/notify2</t>
@@ -1891,10 +2015,24 @@
 </t>
         </is>
       </c>
-      <c r="K27" s="47" t="n"/>
-      <c r="L27" s="15" t="n"/>
-      <c r="M27" s="44" t="n"/>
-      <c r="N27" s="15" t="n"/>
+      <c r="K27" s="47" t="inlineStr">
+        <is>
+          <t>consent notify 8b741177-6594-4137-b999-149176c60196 GRANTED, consent 6b153ccb, hip IN3610001937; on-notify OK accepted; HI request fa855d87-9ff0-4c50-b124-a076ee45b167 (dataPushUrl, keyMaterial ECDH curve25519 with nonce); on-request ACKNOWLEDGED accepted; push of WR-2 as application/fhir+json with ECDH/Curve25519 keyMaterial -&gt; 2xx; notify TRANSFERRED with WR-2 DELIVERED accepted (transfer 57); PHR app shows the records decrypted as Prescription record and Clinical consultation report</t>
+        </is>
+      </c>
+      <c r="L27" s="15" t="inlineStr">
+        <is>
+          <t>CONDITIONAL PASS</t>
+        </is>
+      </c>
+      <c r="M27" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="N27" s="15" t="inlineStr">
+        <is>
+          <t>Expected Result met: records received in the PHR app, decrypted with the HIP's public key and nonce, in NRCES document types (tester's screenshots phr-1..3; records also delivered by transfers 51 and 53 this run). Pushed care contexts are within the consent's and the request date range equals the consent's. Condition: ClinicX has no screen that shows the stored consent (HI types, date range, purpose, expiry); it is stored whole in AbdmConsents only. Outbound bodies are not stored by the build. Extra check (revocation) not run. Evidence 1.txt, phr-1..3.</t>
+        </is>
+      </c>
       <c r="O27" s="57" t="inlineStr">
         <is>
           <r>

</xml_diff>

<commit_message>
chore(abdm-ft): HIP_INIT_SHARE_CARECONTEXT passes on re-run; M2 report 13 of 13 PASS
HIP_INIT_SHARE_CARECONTEXT was a conditional pass on 85ae1bd because no
ClinicX screen showed the stored consent. Re-run on 2026-10-29 with the
tester on backend db30fa2 / frontend feb708f, after the Consents view was
added: consent 023332f4 GRANTED, notify 8b0b8f8b, HI request 7a34c022,
transfer 60 DELIVERED, the consent shown under ABDM Records > Consents with
its HI types, date range, purpose and expiry, and the record decrypted in the
PHR app. Workbook rewritten (check exit 0) and report rebuilt: 13 PASS, no
conditional pass. Run log, manifest, meta (builds, finding, re-run note) and
the plan updated; the earlier evidence and final files are kept in archive/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/abdm-ft/final/M2_BUILDING_HIP_TEST_CASES.xlsx
+++ b/abdm-ft/final/M2_BUILDING_HIP_TEST_CASES.xlsx
@@ -865,7 +865,7 @@
     <row r="5">
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Application/ System Name: ClinicX (Yira Health Tech) - HIP IN3610001937 Ocimum dentistry; backend 85ae1bd, frontend ab5a8a0</t>
+          <t>Application/ System Name: ClinicX web (HIP IN3610001937, Ocimum dentistry)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -2017,20 +2017,20 @@
       </c>
       <c r="K27" s="47" t="inlineStr">
         <is>
-          <t>consent notify 8b741177-6594-4137-b999-149176c60196 GRANTED, consent 6b153ccb, hip IN3610001937; on-notify OK accepted; HI request fa855d87-9ff0-4c50-b124-a076ee45b167 (dataPushUrl, keyMaterial ECDH curve25519 with nonce); on-request ACKNOWLEDGED accepted; push of WR-2 as application/fhir+json with ECDH/Curve25519 keyMaterial -&gt; 2xx; notify TRANSFERRED with WR-2 DELIVERED accepted (transfer 57); PHR app shows the records decrypted as Prescription record and Clinical consultation report</t>
+          <t>consent notify 8b0b8f8b-2d65-4296-9c59-6865556cd787 GRANTED, consent 023332f4, hip IN3610001937; on-notify OK accepted; HI request 7a34c022-ec56-46d6-a0dc-2fc139eb86c6 (transaction a5f7b891, dataPushUrl, keyMaterial ECDH curve25519 with nonce); on-request ACKNOWLEDGED accepted; push of RX-D7CD5098 as application/fhir+json with ECDH/Curve25519 keyMaterial -&gt; 2xx; notify TRANSFERRED with RX-D7CD5098 DELIVERED accepted (transfer 60); Screen: ABDM Records &gt; Consents shows the consent Granted, Self Requested, its 8 HI types, Records dated 29 Oct 1926 to 29 Oct 2026, Expiry 29 Oct 2126, 1 delivered; PHR app shows the Prescription record decrypted</t>
         </is>
       </c>
       <c r="L27" s="15" t="inlineStr">
         <is>
-          <t>CONDITIONAL PASS</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M27" s="44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N27" s="15" t="inlineStr">
         <is>
-          <t>Expected Result met: records received in the PHR app, decrypted with the HIP's public key and nonce, in NRCES document types (tester's screenshots phr-1..3; records also delivered by transfers 51 and 53 this run). Pushed care contexts are within the consent's and the request date range equals the consent's. Condition: ClinicX has no screen that shows the stored consent (HI types, date range, purpose, expiry); it is stored whole in AbdmConsents only. Outbound bodies are not stored by the build. Extra check (revocation) not run. Evidence 1.txt, phr-1..3.</t>
+          <t>Expected Result met on backend db30fa2 / frontend feb708f: the record was received in the PHR app, decrypted, as the NRCES Prescription record (phr-1). ClinicX shows the stored consent against the patient under ABDM Records &gt; Consents, with its HI types, date range, purpose and expiry and what was sent under it (1). The pushed care context is within the consent's, and the request date range equals the consent's. Re-run on 2026-10-29: the 2026-10-28 pass on 85ae1bd was a conditional pass because no screen showed the stored consent; the Consents view was added since. Pass 1 (08:35) met the exit condition, but the view showed its times 5h30 early; fixed in db30fa2 and pass 2 (08:50) recorded. Outbound bodies are not stored by the build. Extra check (revocation) not run. Evidence 1.png, 1.txt, flow.txt, phr-1.png.</t>
         </is>
       </c>
       <c r="O27" s="57" t="inlineStr">

</xml_diff>

<commit_message>
chore(abdm-ft): name the product Yira Clinics in the M2 report
The report, workbook, results and meta now use the product name, and the
report is version 1.1. A note in the report says the screens still show
the working name ClinicX. The build details keep the repository names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/abdm-ft/final/M2_BUILDING_HIP_TEST_CASES.xlsx
+++ b/abdm-ft/final/M2_BUILDING_HIP_TEST_CASES.xlsx
@@ -865,7 +865,7 @@
     <row r="5">
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Application/ System Name: ClinicX web (HIP IN3610001937, Ocimum dentistry)</t>
+          <t>Application/ System Name: Yira Clinics web (HIP IN3610001937, Ocimum dentistry)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -1727,7 +1727,7 @@
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="16" t="inlineStr">
         <is>
-          <t>init 764fd0a5-cd3f-4b0d-8e1c-038a56341033 (transactionId f3c99f71, selected RX-67209C38) -&gt; on-init with link.referenceNumber a402340b-c3d4-420f-88bb-26b0ca563e4d, authenticationType DIRECT, communicationMedium MOBILE, accepted; OTP sent by the HIP (ClinicX SMS) to the mobile ending 5506; confirm 44b6d7d6-9720-4573-b350-b65c8cf57e9d with confirmation.linkRefNumber a402340b and token present -&gt; OTP verified, on-confirm with RX-67209C38 only, accepted; care context linked via patient to xxx0606@sbx</t>
+          <t>init 764fd0a5-cd3f-4b0d-8e1c-038a56341033 (transactionId f3c99f71, selected RX-67209C38) -&gt; on-init with link.referenceNumber a402340b-c3d4-420f-88bb-26b0ca563e4d, authenticationType DIRECT, communicationMedium MOBILE, accepted; OTP sent by the HIP (Yira Clinics SMS) to the mobile ending 5506; confirm 44b6d7d6-9720-4573-b350-b65c8cf57e9d with confirmation.linkRefNumber a402340b and token present -&gt; OTP verified, on-confirm with RX-67209C38 only, accepted; care context linked via patient to xxx0606@sbx</t>
         </is>
       </c>
       <c r="L22" s="16" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="N27" s="15" t="inlineStr">
         <is>
-          <t>Expected Result met on backend db30fa2 / frontend feb708f: the record was received in the PHR app, decrypted, as the NRCES Prescription record (phr-1). ClinicX shows the stored consent against the patient under ABDM Records &gt; Consents, with its HI types, date range, purpose and expiry and what was sent under it (1). The pushed care context is within the consent's, and the request date range equals the consent's. Re-run on 2026-10-29: the 2026-10-28 pass on 85ae1bd was a conditional pass because no screen showed the stored consent; the Consents view was added since. Pass 1 (08:35) met the exit condition, but the view showed its times 5h30 early; fixed in db30fa2 and pass 2 (08:50) recorded. Outbound bodies are not stored by the build. Extra check (revocation) not run. Evidence 1.png, 1.txt, flow.txt, phr-1.png.</t>
+          <t>Expected Result met on backend db30fa2 / frontend feb708f: the record was received in the PHR app, decrypted, as the NRCES Prescription record (phr-1). Yira Clinics shows the stored consent against the patient under ABDM Records &gt; Consents, with its HI types, date range, purpose and expiry and what was sent under it (1). The pushed care context is within the consent's, and the request date range equals the consent's. Re-run on 2026-10-29: the 2026-10-28 pass on 85ae1bd was a conditional pass because no screen showed the stored consent; the Consents view was added since. Pass 1 (08:35) met the exit condition, but the view showed its times 5h30 early; fixed in db30fa2 and pass 2 (08:50) recorded. Outbound bodies are not stored by the build. Extra check (revocation) not run. Evidence 1.png, 1.txt, flow.txt, phr-1.png.</t>
         </is>
       </c>
       <c r="O27" s="57" t="inlineStr">

</xml_diff>